<commit_message>
Added template for single month export
</commit_message>
<xml_diff>
--- a/backend/comwrap/resources/excel-templates/forecast-template.xlsx
+++ b/backend/comwrap/resources/excel-templates/forecast-template.xlsx
@@ -5,15 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ozias.as/Desktop/uni/yr 3 (2025-2026)/PSD-TP/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ozias.as/Desktop/uni/yr 3 (2025-2026)/PSD-TP/sh09-main/backend/comwrap/resources/excel-templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73ACC67F-940C-464F-8A83-740D014C8E7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB5D6045-DB11-D041-8C80-CA46109812AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17220" xr2:uid="{4108D922-1C2C-8F45-B11F-7B4A4E310542}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17220" activeTab="1" xr2:uid="{4108D922-1C2C-8F45-B11F-7B4A4E310542}"/>
   </bookViews>
   <sheets>
-    <sheet name="Resource Allocation" sheetId="1" r:id="rId1"/>
+    <sheet name="Multi-Month Template" sheetId="3" r:id="rId1"/>
+    <sheet name="Single Month Template" sheetId="1" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="39">
   <si>
     <t>Resource Allocation</t>
   </si>
@@ -141,6 +143,15 @@
   </si>
   <si>
     <t>TOTAL - LName, Fname</t>
+  </si>
+  <si>
+    <t>Single month resource allocation (HYPO/Work)</t>
+  </si>
+  <si>
+    <t>Days Allocated</t>
+  </si>
+  <si>
+    <t>Hours Allocated</t>
   </si>
 </sst>
 </file>
@@ -575,7 +586,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="24">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -864,6 +875,30 @@
       <right/>
       <top style="thin">
         <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -914,7 +949,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -990,6 +1025,10 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="22" xfId="42" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="20" fillId="37" borderId="17" xfId="42" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="23" xfId="42" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="38" borderId="13" xfId="42" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="16" xfId="42" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="27" fillId="33" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -999,8 +1038,24 @@
     <xf numFmtId="0" fontId="20" fillId="38" borderId="11" xfId="42" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="38" borderId="13" xfId="42" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="38" borderId="12" xfId="42" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="16" xfId="42" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="42" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="33" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="11" xfId="42" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="12" xfId="42" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="24" xfId="42" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="17" xfId="42" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -1377,7 +1432,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8A2FCBC-C538-FE4C-A033-B4F764A737FB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FEF80BD-A2BA-C44B-985E-5D2CCDC15C11}">
   <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1566,10 +1621,10 @@
       <c r="H18" s="17"/>
       <c r="I18" s="17"/>
       <c r="J18" s="17"/>
-      <c r="K18" s="36" t="s">
+      <c r="K18" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="L18" s="31" t="s">
+      <c r="L18" s="33" t="s">
         <v>24</v>
       </c>
       <c r="M18" s="18"/>
@@ -1602,7 +1657,7 @@
         <v>32</v>
       </c>
       <c r="K19" s="23"/>
-      <c r="L19" s="32"/>
+      <c r="L19" s="34"/>
     </row>
     <row r="20" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="24" t="s">
@@ -1627,17 +1682,17 @@
     </row>
     <row r="21" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="28"/>
-      <c r="B21" s="33" t="s">
+      <c r="B21" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="C21" s="34"/>
-      <c r="D21" s="34"/>
-      <c r="E21" s="34"/>
-      <c r="F21" s="34"/>
-      <c r="G21" s="34"/>
-      <c r="H21" s="34"/>
-      <c r="I21" s="34"/>
-      <c r="J21" s="35"/>
+      <c r="C21" s="36"/>
+      <c r="D21" s="36"/>
+      <c r="E21" s="36"/>
+      <c r="F21" s="36"/>
+      <c r="G21" s="36"/>
+      <c r="H21" s="36"/>
+      <c r="I21" s="36"/>
+      <c r="J21" s="37"/>
       <c r="K21" s="29">
         <f t="shared" ref="K21" si="0">SUM(K20:K20)</f>
         <v>0</v>
@@ -1651,4 +1706,301 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8A2FCBC-C538-FE4C-A033-B4F764A737FB}">
+  <dimension ref="A1:N21"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="16.5" style="2" customWidth="1"/>
+    <col min="2" max="6" width="12.5" style="2" customWidth="1"/>
+    <col min="7" max="7" width="3.33203125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="3.33203125" style="3" customWidth="1"/>
+    <col min="9" max="9" width="16" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="62.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.83203125" style="2" customWidth="1"/>
+    <col min="12" max="12" width="15.83203125" style="2" customWidth="1"/>
+    <col min="13" max="13" width="4.33203125" style="2" customWidth="1"/>
+    <col min="14" max="16384" width="10.83203125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="38"/>
+    </row>
+    <row r="3" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="8"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+    </row>
+    <row r="4" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+    </row>
+    <row r="6" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
+    </row>
+    <row r="7" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+    </row>
+    <row r="8" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+    </row>
+    <row r="9" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+    </row>
+    <row r="10" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" s="11"/>
+    </row>
+    <row r="11" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" s="11"/>
+    </row>
+    <row r="12" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+    </row>
+    <row r="13" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+    </row>
+    <row r="14" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="12"/>
+      <c r="C14" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H14" s="13"/>
+    </row>
+    <row r="15" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="7"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H15" s="13"/>
+    </row>
+    <row r="16" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="7"/>
+      <c r="B16" s="15"/>
+      <c r="C16" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H16" s="13"/>
+    </row>
+    <row r="17" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="7"/>
+      <c r="B17" s="16"/>
+      <c r="C17" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="13"/>
+      <c r="H17" s="2"/>
+    </row>
+    <row r="18" spans="1:14" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="17"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="17"/>
+      <c r="I18" s="17"/>
+      <c r="J18" s="17"/>
+      <c r="K18" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="L18" s="41"/>
+      <c r="M18" s="39" t="s">
+        <v>24</v>
+      </c>
+      <c r="N18" s="18"/>
+    </row>
+    <row r="19" spans="1:14" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="D19" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="E19" s="21" t="s">
+        <v>29</v>
+      </c>
+      <c r="F19" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="G19" s="20"/>
+      <c r="H19" s="20"/>
+      <c r="I19" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="J19" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="K19" s="42" t="s">
+        <v>37</v>
+      </c>
+      <c r="L19" s="43" t="s">
+        <v>38</v>
+      </c>
+      <c r="M19" s="34"/>
+    </row>
+    <row r="20" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" s="25"/>
+      <c r="C20" s="25"/>
+      <c r="D20" s="25"/>
+      <c r="E20" s="25"/>
+      <c r="F20" s="25"/>
+      <c r="G20" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="H20" s="25"/>
+      <c r="I20" s="25"/>
+      <c r="J20" s="25"/>
+      <c r="K20" s="25"/>
+      <c r="L20" s="26">
+        <v>0</v>
+      </c>
+      <c r="M20" s="27"/>
+      <c r="N20" s="18"/>
+    </row>
+    <row r="21" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="28"/>
+      <c r="B21" s="35" t="s">
+        <v>35</v>
+      </c>
+      <c r="C21" s="36"/>
+      <c r="D21" s="36"/>
+      <c r="E21" s="36"/>
+      <c r="F21" s="36"/>
+      <c r="G21" s="36"/>
+      <c r="H21" s="36"/>
+      <c r="I21" s="36"/>
+      <c r="J21" s="37"/>
+      <c r="K21" s="31"/>
+      <c r="L21" s="29">
+        <f t="shared" ref="L21" si="0">SUM(L20:L20)</f>
+        <v>0</v>
+      </c>
+      <c r="M21" s="30"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="M18:M19"/>
+    <mergeCell ref="B21:J21"/>
+    <mergeCell ref="K18:L18"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D21AA24-EDA7-6643-A3BB-79BDD3FEEBED}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
updated routes and added helper functions in backend
</commit_message>
<xml_diff>
--- a/backend/comwrap/resources/excel-templates/forecast-template.xlsx
+++ b/backend/comwrap/resources/excel-templates/forecast-template.xlsx
@@ -8,14 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ozias.as/Desktop/uni/yr 3 (2025-2026)/PSD-TP/sh09-main/backend/comwrap/resources/excel-templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB5D6045-DB11-D041-8C80-CA46109812AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9F56FA3-CAC6-B946-BBB2-93844D7D8B75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17220" activeTab="1" xr2:uid="{4108D922-1C2C-8F45-B11F-7B4A4E310542}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17220" xr2:uid="{4108D922-1C2C-8F45-B11F-7B4A4E310542}"/>
   </bookViews>
   <sheets>
     <sheet name="Multi-Month Template" sheetId="3" r:id="rId1"/>
     <sheet name="Single Month Template" sheetId="1" r:id="rId2"/>
-    <sheet name="Sheet1" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -949,7 +948,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -1029,19 +1028,24 @@
     <xf numFmtId="0" fontId="19" fillId="33" borderId="16" xfId="42" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="38" borderId="11" xfId="42" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="38" borderId="12" xfId="42" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="42" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="24" xfId="42" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="17" xfId="42" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="27" fillId="33" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="33" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="38" borderId="11" xfId="42" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="38" borderId="13" xfId="42" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="38" borderId="12" xfId="42" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="42" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="27" fillId="33" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -1050,12 +1054,6 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="33" borderId="12" xfId="42" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="24" xfId="42" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="17" xfId="42" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -1624,7 +1622,7 @@
       <c r="K18" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="L18" s="33" t="s">
+      <c r="L18" s="38" t="s">
         <v>24</v>
       </c>
       <c r="M18" s="18"/>
@@ -1657,7 +1655,7 @@
         <v>32</v>
       </c>
       <c r="K19" s="23"/>
-      <c r="L19" s="34"/>
+      <c r="L19" s="39"/>
     </row>
     <row r="20" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="24" t="s">
@@ -1682,17 +1680,17 @@
     </row>
     <row r="21" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="28"/>
-      <c r="B21" s="35" t="s">
+      <c r="B21" s="33" t="s">
         <v>35</v>
       </c>
-      <c r="C21" s="36"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="36"/>
-      <c r="F21" s="36"/>
-      <c r="G21" s="36"/>
-      <c r="H21" s="36"/>
-      <c r="I21" s="36"/>
-      <c r="J21" s="37"/>
+      <c r="C21" s="31"/>
+      <c r="D21" s="31"/>
+      <c r="E21" s="31"/>
+      <c r="F21" s="31"/>
+      <c r="G21" s="31"/>
+      <c r="H21" s="31"/>
+      <c r="I21" s="31"/>
+      <c r="J21" s="34"/>
       <c r="K21" s="29">
         <f t="shared" ref="K21" si="0">SUM(K20:K20)</f>
         <v>0</v>
@@ -1700,9 +1698,8 @@
       <c r="L21" s="30"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="L18:L19"/>
-    <mergeCell ref="B21:J21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1738,7 +1735,7 @@
       <c r="H1" s="5"/>
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
-      <c r="K1" s="38"/>
+      <c r="K1" s="35"/>
     </row>
     <row r="3" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
@@ -1900,11 +1897,11 @@
       <c r="H18" s="17"/>
       <c r="I18" s="17"/>
       <c r="J18" s="17"/>
-      <c r="K18" s="40" t="s">
+      <c r="K18" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="L18" s="41"/>
-      <c r="M18" s="39" t="s">
+      <c r="L18" s="42"/>
+      <c r="M18" s="40" t="s">
         <v>24</v>
       </c>
       <c r="N18" s="18"/>
@@ -1936,13 +1933,13 @@
       <c r="J19" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="K19" s="42" t="s">
+      <c r="K19" s="36" t="s">
         <v>37</v>
       </c>
-      <c r="L19" s="43" t="s">
+      <c r="L19" s="37" t="s">
         <v>38</v>
       </c>
-      <c r="M19" s="34"/>
+      <c r="M19" s="39"/>
     </row>
     <row r="20" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="24" t="s">
@@ -1968,17 +1965,17 @@
     </row>
     <row r="21" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="28"/>
-      <c r="B21" s="35" t="s">
+      <c r="B21" s="33" t="s">
         <v>35</v>
       </c>
-      <c r="C21" s="36"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="36"/>
-      <c r="F21" s="36"/>
-      <c r="G21" s="36"/>
-      <c r="H21" s="36"/>
-      <c r="I21" s="36"/>
-      <c r="J21" s="37"/>
+      <c r="C21" s="31"/>
+      <c r="D21" s="31"/>
+      <c r="E21" s="31"/>
+      <c r="F21" s="31"/>
+      <c r="G21" s="31"/>
+      <c r="H21" s="31"/>
+      <c r="I21" s="31"/>
+      <c r="J21" s="34"/>
       <c r="K21" s="31"/>
       <c r="L21" s="29">
         <f t="shared" ref="L21" si="0">SUM(L20:L20)</f>
@@ -1987,20 +1984,10 @@
       <c r="M21" s="30"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="M18:M19"/>
-    <mergeCell ref="B21:J21"/>
     <mergeCell ref="K18:L18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D21AA24-EDA7-6643-A3BB-79BDD3FEEBED}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>